<commit_message>
Major change, upgrade pics
</commit_message>
<xml_diff>
--- a/hw3/result/nn_performance_with_clusters_comparison.xlsx
+++ b/hw3/result/nn_performance_with_clusters_comparison.xlsx
@@ -483,7 +483,7 @@
         <v>0.9824561403508771</v>
       </c>
       <c r="D2" t="n">
-        <v>568.5337722301483</v>
+        <v>847.3920893669128</v>
       </c>
       <c r="E2" t="n">
         <v>0.9824561403508771</v>
@@ -511,7 +511,7 @@
         <v>0.9824561403508771</v>
       </c>
       <c r="D3" t="n">
-        <v>571.911187171936</v>
+        <v>1066.765557289124</v>
       </c>
       <c r="E3" t="n">
         <v>0.9824561403508771</v>
@@ -539,7 +539,7 @@
         <v>0.9736842105263158</v>
       </c>
       <c r="D4" t="n">
-        <v>596.4928507804871</v>
+        <v>1033.354111909866</v>
       </c>
       <c r="E4" t="n">
         <v>0.9737190197716513</v>

</xml_diff>